<commit_message>
Fix fallback scoring to require same-round evidence, add elimination check, and read predicted 3rd place/champion directly from Excel honor board
- Individual-team fallback now requires the team to win (or tie and reappear) within the same round bucket as the real match, not just anywhere in the bracket
- Split 3rd place (103) and final (104) into separate round buckets since they are alternative outcomes of the semifinal, not a progression
- Read Campeón/Subcampeón/3º puesto directly from each participant's WORLDCUP sheet for tie-break display on IDs 103/104 instead of inferring it
- Add regression tests for the new same-round rule

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clasificacion.xlsx
+++ b/clasificacion.xlsx
@@ -480,7 +480,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D2" t="n">
         <v>16</v>
@@ -492,7 +492,7 @@
         <v>108</v>
       </c>
       <c r="G2" t="n">
-        <v>343</v>
+        <v>333</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D3" t="n">
         <v>11</v>
@@ -522,7 +522,7 @@
         <v>93</v>
       </c>
       <c r="G3" t="n">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -540,7 +540,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D4" t="n">
         <v>16</v>
@@ -552,7 +552,7 @@
         <v>96</v>
       </c>
       <c r="G4" t="n">
-        <v>329</v>
+        <v>319</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D5" t="n">
         <v>8</v>
@@ -582,7 +582,7 @@
         <v>81</v>
       </c>
       <c r="G5" t="n">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -600,7 +600,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D6" t="n">
         <v>9</v>
@@ -612,7 +612,7 @@
         <v>87</v>
       </c>
       <c r="G6" t="n">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -630,7 +630,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D7" t="n">
         <v>11</v>
@@ -642,7 +642,7 @@
         <v>102</v>
       </c>
       <c r="G7" t="n">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -656,23 +656,23 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Sergio_Fernandez</t>
+          <t>Raúl_Canabal</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D8" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F8" t="n">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="G8" t="n">
-        <v>314</v>
+        <v>305</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -686,23 +686,23 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Raúl_Canabal</t>
+          <t>Sergio_Fernandez</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D9" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F9" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="G9" t="n">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -720,7 +720,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D10" t="n">
         <v>12</v>
@@ -732,7 +732,7 @@
         <v>96</v>
       </c>
       <c r="G10" t="n">
-        <v>307</v>
+        <v>297</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -750,7 +750,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D11" t="n">
         <v>9</v>
@@ -762,7 +762,7 @@
         <v>81</v>
       </c>
       <c r="G11" t="n">
-        <v>307</v>
+        <v>297</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -776,23 +776,23 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Alberto_Martin_Lopez</t>
+          <t>Nessi_Morant</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D12" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F12" t="n">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="G12" t="n">
-        <v>306</v>
+        <v>292</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -806,23 +806,23 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Nessi_Morant</t>
+          <t>Alberto_Martin_Lopez</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D13" t="n">
+        <v>7</v>
+      </c>
+      <c r="E13" t="n">
         <v>10</v>
       </c>
-      <c r="E13" t="n">
-        <v>11</v>
-      </c>
       <c r="F13" t="n">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="G13" t="n">
-        <v>302</v>
+        <v>291</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -836,23 +836,23 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Alberto_Villardón</t>
+          <t>Jorge_Gamero</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="D14" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E14" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F14" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G14" t="n">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -866,23 +866,23 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Jesús_García</t>
+          <t>Cristian_Luque</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="D15" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E15" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F15" t="n">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="G15" t="n">
-        <v>298</v>
+        <v>284</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -896,23 +896,23 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Jorge_Gamero</t>
+          <t>Alberto_Villardón</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="D16" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E16" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F16" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="G16" t="n">
-        <v>295</v>
+        <v>283</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -926,23 +926,23 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Cristian_Luque</t>
+          <t>Jesús_García</t>
         </is>
       </c>
       <c r="C17" t="n">
         <v>40</v>
       </c>
       <c r="D17" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E17" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F17" t="n">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="G17" t="n">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D18" t="n">
         <v>8</v>
@@ -972,7 +972,7 @@
         <v>84</v>
       </c>
       <c r="G18" t="n">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -990,7 +990,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D19" t="n">
         <v>8</v>
@@ -1002,7 +1002,7 @@
         <v>81</v>
       </c>
       <c r="G19" t="n">
-        <v>285</v>
+        <v>270</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1020,7 +1020,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D20" t="n">
         <v>8</v>
@@ -1032,7 +1032,7 @@
         <v>87</v>
       </c>
       <c r="G20" t="n">
-        <v>278</v>
+        <v>268</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1046,23 +1046,23 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Javier_García</t>
+          <t>Samuel_Fernández_Duarte</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D21" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F21" t="n">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="G21" t="n">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1076,23 +1076,23 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Juan_Carlos_Ruiz</t>
+          <t>Óscar_Espinosa</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D22" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E22" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F22" t="n">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="G22" t="n">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1106,23 +1106,23 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Óscar_Espinosa</t>
+          <t>Juan_Carlos_Ruiz</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D23" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F23" t="n">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="G23" t="n">
-        <v>268</v>
+        <v>259</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1140,7 +1140,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D24" t="n">
         <v>6</v>
@@ -1152,7 +1152,7 @@
         <v>81</v>
       </c>
       <c r="G24" t="n">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D25" t="n">
         <v>10</v>
@@ -1182,7 +1182,7 @@
         <v>78</v>
       </c>
       <c r="G25" t="n">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -1196,23 +1196,23 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Samuel_Fernández_Duarte</t>
+          <t>Javier_García</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D26" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F26" t="n">
-        <v>96</v>
+        <v>75</v>
       </c>
       <c r="G26" t="n">
-        <v>264</v>
+        <v>252</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -1230,7 +1230,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D27" t="n">
         <v>8</v>
@@ -1242,7 +1242,7 @@
         <v>87</v>
       </c>
       <c r="G27" t="n">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -1260,7 +1260,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D28" t="n">
         <v>10</v>
@@ -1272,7 +1272,7 @@
         <v>57</v>
       </c>
       <c r="G28" t="n">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix Bota de Oro / Balón de Oro scoring and silence harmless openpyxl warnings
- The "Datos" sheet's PREMIO column only ever held the category label ("Bota de oro"),
  never the participant's actual player prediction, so this bonus never scored correctly.
  The real prediction lives in each participant's WORLDCUP sheet "Cuadro de honor".
- Read Bota de Oro / Balón de Oro (and reuse Campeón/Subcampeón/3º puesto) from that
  sheet via leer_cuadro_honor() instead of the broken "Datos" column.
- Compare player names accent-insensitively and allow full name vs surname-only
  predictions to match (e.g. "Kylian Mbappe" / "Mbappé" / "Mbappe" all count).
- Suppress openpyxl's harmless "extension not supported" warnings when reading the
  heavily-formatted WORLDCUP sheet.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clasificacion.xlsx
+++ b/clasificacion.xlsx
@@ -476,27 +476,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Noel_Olivares</t>
+          <t>David_De_Paz</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D2" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F2" t="n">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="G2" t="n">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>&lt;span style='color:#ffffff; font-weight:bold'&gt;=&lt;/span&gt;</t>
+          <t>&lt;span style='color:#00ff00'&gt;⬆️ +1&lt;/span&gt;</t>
         </is>
       </c>
     </row>
@@ -506,27 +506,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>David_De_Paz</t>
+          <t>Noel_Olivares</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D3" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="E3" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F3" t="n">
-        <v>93</v>
+        <v>108</v>
       </c>
       <c r="G3" t="n">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>&lt;span style='color:#ffffff; font-weight:bold'&gt;=&lt;/span&gt;</t>
+          <t>&lt;span style='color:#ff4d4d'&gt;⬇️ -1&lt;/span&gt;</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>&lt;span style='color:#00ff00'&gt;⬆️ +1&lt;/span&gt;</t>
+          <t>&lt;span style='color:#ffffff; font-weight:bold'&gt;=&lt;/span&gt;</t>
         </is>
       </c>
     </row>
@@ -586,7 +586,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>&lt;span style='color:#ff4d4d'&gt;⬇️ -1&lt;/span&gt;</t>
+          <t>&lt;span style='color:#ffffff; font-weight:bold'&gt;=&lt;/span&gt;</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>&lt;span style='color:#00ff00'&gt;⬆️ +1&lt;/span&gt;</t>
+          <t>&lt;span style='color:#ffffff; font-weight:bold'&gt;=&lt;/span&gt;</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>&lt;span style='color:#ff4d4d'&gt;⬇️ -1&lt;/span&gt;</t>
+          <t>&lt;span style='color:#ffffff; font-weight:bold'&gt;=&lt;/span&gt;</t>
         </is>
       </c>
     </row>
@@ -716,27 +716,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alvaro_Terron</t>
+          <t>Javier_Leton</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="D10" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E10" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="F10" t="n">
-        <v>81</v>
+        <v>106</v>
       </c>
       <c r="G10" t="n">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>&lt;span style='color:#00ff00'&gt;⬆️ +1&lt;/span&gt;</t>
+          <t>&lt;span style='color:#ffffff; font-weight:bold'&gt;=&lt;/span&gt;</t>
         </is>
       </c>
     </row>
@@ -759,14 +759,14 @@
         <v>11</v>
       </c>
       <c r="F11" t="n">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="G11" t="n">
-        <v>297</v>
+        <v>307</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>&lt;span style='color:#00ff00'&gt;⬆️ +1&lt;/span&gt;</t>
+          <t>&lt;span style='color:#ffffff; font-weight:bold'&gt;=&lt;/span&gt;</t>
         </is>
       </c>
     </row>
@@ -776,27 +776,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Javier_Leton</t>
+          <t>Cristian_Luque</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D12" t="n">
         <v>12</v>
       </c>
       <c r="E12" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F12" t="n">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="G12" t="n">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>&lt;span style='color:#ff4d4d'&gt;⬇️ -2&lt;/span&gt;</t>
+          <t>&lt;span style='color:#ffffff; font-weight:bold'&gt;=&lt;/span&gt;</t>
         </is>
       </c>
     </row>
@@ -806,27 +806,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Jorge_Gamero</t>
+          <t>Alvaro_Terron</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D13" t="n">
+        <v>9</v>
+      </c>
+      <c r="E13" t="n">
         <v>14</v>
       </c>
-      <c r="E13" t="n">
-        <v>8</v>
-      </c>
       <c r="F13" t="n">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="G13" t="n">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>&lt;span style='color:#00ff00'&gt;⬆️ +1&lt;/span&gt;</t>
+          <t>&lt;span style='color:#ffffff; font-weight:bold'&gt;=&lt;/span&gt;</t>
         </is>
       </c>
     </row>
@@ -836,27 +836,27 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cristian_Luque</t>
+          <t>Alberto_Martin_Lopez</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D14" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E14" t="n">
         <v>10</v>
       </c>
       <c r="F14" t="n">
-        <v>81</v>
+        <v>109</v>
       </c>
       <c r="G14" t="n">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>&lt;span style='color:#00ff00'&gt;⬆️ +1&lt;/span&gt;</t>
+          <t>&lt;span style='color:#00ff00'&gt;⬆️ +2&lt;/span&gt;</t>
         </is>
       </c>
     </row>
@@ -866,27 +866,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Alberto_Martin_Lopez</t>
+          <t>Jesús_García</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D15" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F15" t="n">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="G15" t="n">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>&lt;span style='color:#ff4d4d'&gt;⬇️ -2&lt;/span&gt;</t>
+          <t>&lt;span style='color:#00ff00'&gt;⬆️ +2&lt;/span&gt;</t>
         </is>
       </c>
     </row>
@@ -909,14 +909,14 @@
         <v>12</v>
       </c>
       <c r="F16" t="n">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="G16" t="n">
-        <v>288</v>
+        <v>298</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>&lt;span style='color:#ffffff; font-weight:bold'&gt;=&lt;/span&gt;</t>
+          <t>&lt;span style='color:#ff4d4d'&gt;⬇️ -2&lt;/span&gt;</t>
         </is>
       </c>
     </row>
@@ -926,27 +926,27 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Jesús_García</t>
+          <t>Jorge_Gamero</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D17" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E17" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F17" t="n">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="G17" t="n">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>&lt;span style='color:#ffffff; font-weight:bold'&gt;=&lt;/span&gt;</t>
+          <t>&lt;span style='color:#ff4d4d'&gt;⬇️ -2&lt;/span&gt;</t>
         </is>
       </c>
     </row>
@@ -969,10 +969,10 @@
         <v>8</v>
       </c>
       <c r="F18" t="n">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="G18" t="n">
-        <v>276</v>
+        <v>286</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1016,27 +1016,27 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Óscar_Espinosa</t>
+          <t>Javier_Sánchez_Moreno</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="D20" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E20" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F20" t="n">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="G20" t="n">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>&lt;span style='color:#00ff00'&gt;⬆️ +2&lt;/span&gt;</t>
+          <t>&lt;span style='color:#00ff00'&gt;⬆️ +5&lt;/span&gt;</t>
         </is>
       </c>
     </row>
@@ -1046,20 +1046,20 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Ruth_Galvin</t>
+          <t>Óscar_Espinosa</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D21" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="E21" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F21" t="n">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="G21" t="n">
         <v>268</v>
@@ -1076,23 +1076,23 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Samuel_Fernández_Duarte</t>
+          <t>Ruth_Galvin</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D22" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E22" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F22" t="n">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="G22" t="n">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1106,27 +1106,27 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Javier_Sánchez_Moreno</t>
+          <t>Javier_García</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D23" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E23" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F23" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="G23" t="n">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>&lt;span style='color:#00ff00'&gt;⬆️ +1&lt;/span&gt;</t>
+          <t>&lt;span style='color:#ff4d4d'&gt;⬇️ -1&lt;/span&gt;</t>
         </is>
       </c>
     </row>
@@ -1136,27 +1136,27 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Juan_Carlos_Ruiz</t>
+          <t>Samuel_Fernández_Duarte</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D24" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E24" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F24" t="n">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="G24" t="n">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>&lt;span style='color:#ff4d4d'&gt;⬇️ -1&lt;/span&gt;</t>
+          <t>&lt;span style='color:#ffffff; font-weight:bold'&gt;=&lt;/span&gt;</t>
         </is>
       </c>
     </row>
@@ -1166,27 +1166,27 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Javier_García</t>
+          <t>Ángel_Gutiérrez</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D25" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E25" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F25" t="n">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="G25" t="n">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>&lt;span style='color:#00ff00'&gt;⬆️ +1&lt;/span&gt;</t>
+          <t>&lt;span style='color:#ff4d4d'&gt;⬇️ -2&lt;/span&gt;</t>
         </is>
       </c>
     </row>
@@ -1196,27 +1196,27 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Ángel_Gutiérrez</t>
+          <t>Juan_Carlos_Ruiz</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D26" t="n">
         <v>10</v>
       </c>
       <c r="E26" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F26" t="n">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="G26" t="n">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>&lt;span style='color:#ff4d4d'&gt;⬇️ -1&lt;/span&gt;</t>
+          <t>&lt;span style='color:#ffffff; font-weight:bold'&gt;=&lt;/span&gt;</t>
         </is>
       </c>
     </row>
@@ -1269,10 +1269,10 @@
         <v>5</v>
       </c>
       <c r="F28" t="n">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="G28" t="n">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>

</xml_diff>